<commit_message>
made two maps (china, europe)
</commit_message>
<xml_diff>
--- a/docs/conquest/bank.xlsx
+++ b/docs/conquest/bank.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\js\games\docs\conquest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DAFCE84-70AD-405B-8A82-2299D9723DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4856BDC7-EBD3-4D94-AF18-511FF3C8DCED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>id</t>
   </si>
@@ -84,16 +84,45 @@
   </si>
   <si>
     <t>SCRIPTjs</t>
+  </si>
+  <si>
+    <t>\text{find\ }\frac{3+2^2}{5}</t>
+  </si>
+  <si>
+    <t>test2</t>
+  </si>
+  <si>
+    <t>find the above</t>
+  </si>
+  <si>
+    <t>\text{find\ }\frac{2+\sqrt{2}}{2-\sqrt{2}}</t>
+  </si>
+  <si>
+    <t>helpjs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -125,9 +154,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -412,6 +443,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="12.6640625" customWidth="1"/>
+    <col min="4" max="4" width="8.88671875" style="1"/>
     <col min="5" max="5" width="16.6640625" customWidth="1"/>
     <col min="6" max="6" width="35.21875" customWidth="1"/>
     <col min="7" max="7" width="59" customWidth="1"/>
@@ -427,7 +459,7 @@
       <c r="C1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E1" t="s">
@@ -447,19 +479,19 @@
       <c r="A2">
         <v>0</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="1">
         <v>4</v>
       </c>
       <c r="E2" t="s">
         <v>3</v>
       </c>
       <c r="G2" t="str">
-        <f>_xlfn.TEXTJOIN($H$7,FALSE,A2:F2)</f>
+        <f>IF(COUNT(B2:F2)&gt;0,_xlfn.TEXTJOIN($H$7,FALSE,A2:F2),"")</f>
         <v>0~~~4~find 2+3-1~</v>
       </c>
       <c r="H2" t="str">
-        <f>_xlfn.TEXTJOIN(H5,FALSE,G2:G4)</f>
-        <v>0~~~4~find 2+3-1~@1~~~0.5~~\text{find}\ \frac{2}3\cdot \frac{6}{8}@2~~test~512~~</v>
+        <f>_xlfn.TEXTJOIN(H5,FALSE,G2:G99)</f>
+        <v>0~~~4~find 2+3-1~@1~~~0.5~~\text{find}\ \frac{2}3\cdot \frac{6}{8}@2~~test~512~~@3~~~1.4~~\text{find\ }\frac{3+2^2}{5}@4~~test2~5.83~~@5~~test2~5.83~find the above~\text{find\ }\frac{2+\sqrt{2}}{2-\sqrt{2}}@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -467,14 +499,14 @@
         <f>A2+1</f>
         <v>1</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="1">
         <v>0.5</v>
       </c>
       <c r="F3" t="s">
         <v>8</v>
       </c>
       <c r="G3" t="str">
-        <f t="shared" ref="G3:G66" si="0">_xlfn.TEXTJOIN($H$7,FALSE,A3:F3)</f>
+        <f t="shared" ref="G3:G66" si="0">IF(COUNT(B3:F3)&gt;0,_xlfn.TEXTJOIN($H$7,FALSE,A3:F3),"")</f>
         <v>1~~~0.5~~\text{find}\ \frac{2}3\cdot \frac{6}{8}</v>
       </c>
     </row>
@@ -486,7 +518,7 @@
       <c r="C4" t="s">
         <v>4</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="1">
         <v>512</v>
       </c>
       <c r="G4" t="str">
@@ -502,9 +534,15 @@
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
+      <c r="D5" s="1">
+        <v>1.4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
       <c r="G5" t="str">
         <f t="shared" si="0"/>
-        <v>3~~~~~</v>
+        <v>3~~~1.4~~\text{find\ }\frac{3+2^2}{5}</v>
       </c>
       <c r="H5" t="s">
         <v>14</v>
@@ -515,9 +553,15 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="1">
+        <v>5.83</v>
+      </c>
       <c r="G6" t="str">
         <f t="shared" si="0"/>
-        <v>4~~~~~</v>
+        <v>4~~test2~5.83~~</v>
       </c>
       <c r="H6" t="s">
         <v>12</v>
@@ -528,9 +572,21 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="1">
+        <v>5.83</v>
+      </c>
+      <c r="E7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" t="s">
+        <v>19</v>
+      </c>
       <c r="G7" t="str">
         <f t="shared" si="0"/>
-        <v>5~~~~~</v>
+        <v>5~~test2~5.83~find the above~\text{find\ }\frac{2+\sqrt{2}}{2-\sqrt{2}}</v>
       </c>
       <c r="H7" t="s">
         <v>13</v>
@@ -543,7 +599,7 @@
       </c>
       <c r="G8" t="str">
         <f t="shared" si="0"/>
-        <v>6~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -553,10 +609,7 @@
       </c>
       <c r="G9" t="str">
         <f t="shared" si="0"/>
-        <v>7~~~~~</v>
-      </c>
-      <c r="H9" t="s">
-        <v>15</v>
+        <v/>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -566,11 +619,7 @@
       </c>
       <c r="G10" t="str">
         <f t="shared" si="0"/>
-        <v>8~~~~~</v>
-      </c>
-      <c r="H10" s="1" t="str">
-        <f>"static raw = String.raw`"&amp;H2&amp;"`"</f>
-        <v>static raw = String.raw`0~~~4~find 2+3-1~@1~~~0.5~~\text{find}\ \frac{2}3\cdot \frac{6}{8}@2~~test~512~~`</v>
+        <v/>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -580,7 +629,7 @@
       </c>
       <c r="G11" t="str">
         <f t="shared" si="0"/>
-        <v>9~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -590,7 +639,10 @@
       </c>
       <c r="G12" t="str">
         <f t="shared" si="0"/>
-        <v>10~~~~~</v>
+        <v/>
+      </c>
+      <c r="H12" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -600,7 +652,11 @@
       </c>
       <c r="G13" t="str">
         <f t="shared" si="0"/>
-        <v>11~~~~~</v>
+        <v/>
+      </c>
+      <c r="H13" s="2" t="str">
+        <f>"static raw = String.raw`"&amp;$H$2</f>
+        <v>static raw = String.raw`0~~~4~find 2+3-1~@1~~~0.5~~\text{find}\ \frac{2}3\cdot \frac{6}{8}@2~~test~512~~@3~~~1.4~~\text{find\ }\frac{3+2^2}{5}@4~~test2~5.83~~@5~~test2~5.83~find the above~\text{find\ }\frac{2+\sqrt{2}}{2-\sqrt{2}}@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@@</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -610,7 +666,7 @@
       </c>
       <c r="G14" t="str">
         <f t="shared" si="0"/>
-        <v>12~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -620,7 +676,7 @@
       </c>
       <c r="G15" t="str">
         <f t="shared" si="0"/>
-        <v>13~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -630,167 +686,174 @@
       </c>
       <c r="G16" t="str">
         <f t="shared" si="0"/>
-        <v>14~~~~~</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="G17" t="str">
         <f t="shared" si="0"/>
-        <v>15~~~~~</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+      <c r="H17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="G18" t="str">
         <f t="shared" si="0"/>
-        <v>16~~~~~</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+      <c r="H18" s="3" t="str">
+        <f>LEFT(H13,FIND("@@", H13)-1)&amp;"`"</f>
+        <v>static raw = String.raw`0~~~4~find 2+3-1~@1~~~0.5~~\text{find}\ \frac{2}3\cdot \frac{6}{8}@2~~test~512~~@3~~~1.4~~\text{find\ }\frac{3+2^2}{5}@4~~test2~5.83~~@5~~test2~5.83~find the above~\text{find\ }\frac{2+\sqrt{2}}{2-\sqrt{2}}`</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="G19" t="str">
         <f t="shared" si="0"/>
-        <v>17~~~~~</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="G20" t="str">
         <f t="shared" si="0"/>
-        <v>18~~~~~</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="G21" t="str">
         <f t="shared" si="0"/>
-        <v>19~~~~~</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="G22" t="str">
         <f t="shared" si="0"/>
-        <v>20~~~~~</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23">
         <f t="shared" si="1"/>
         <v>21</v>
       </c>
       <c r="G23" t="str">
         <f t="shared" si="0"/>
-        <v>21~~~~~</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="G24" t="str">
         <f t="shared" si="0"/>
-        <v>22~~~~~</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
       <c r="G25" t="str">
         <f t="shared" si="0"/>
-        <v>23~~~~~</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="G26" t="str">
         <f t="shared" si="0"/>
-        <v>24~~~~~</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="G27" t="str">
         <f t="shared" si="0"/>
-        <v>25~~~~~</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28">
         <f t="shared" si="1"/>
         <v>26</v>
       </c>
       <c r="G28" t="str">
         <f t="shared" si="0"/>
-        <v>26~~~~~</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29">
         <f t="shared" si="1"/>
         <v>27</v>
       </c>
       <c r="G29" t="str">
         <f t="shared" si="0"/>
-        <v>27~~~~~</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="G30" t="str">
         <f t="shared" si="0"/>
-        <v>28~~~~~</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31">
         <f t="shared" si="1"/>
         <v>29</v>
       </c>
       <c r="G31" t="str">
         <f t="shared" si="0"/>
-        <v>29~~~~~</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
       <c r="G32" t="str">
         <f t="shared" si="0"/>
-        <v>30~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
@@ -800,7 +863,7 @@
       </c>
       <c r="G33" t="str">
         <f t="shared" si="0"/>
-        <v>31~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
@@ -810,7 +873,7 @@
       </c>
       <c r="G34" t="str">
         <f t="shared" si="0"/>
-        <v>32~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
@@ -820,7 +883,7 @@
       </c>
       <c r="G35" t="str">
         <f t="shared" si="0"/>
-        <v>33~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
@@ -830,7 +893,7 @@
       </c>
       <c r="G36" t="str">
         <f t="shared" si="0"/>
-        <v>34~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
@@ -840,7 +903,7 @@
       </c>
       <c r="G37" t="str">
         <f t="shared" si="0"/>
-        <v>35~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
@@ -850,7 +913,7 @@
       </c>
       <c r="G38" t="str">
         <f t="shared" si="0"/>
-        <v>36~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
@@ -860,7 +923,7 @@
       </c>
       <c r="G39" t="str">
         <f t="shared" si="0"/>
-        <v>37~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
@@ -870,7 +933,7 @@
       </c>
       <c r="G40" t="str">
         <f t="shared" si="0"/>
-        <v>38~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
@@ -880,7 +943,7 @@
       </c>
       <c r="G41" t="str">
         <f t="shared" si="0"/>
-        <v>39~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
@@ -890,7 +953,7 @@
       </c>
       <c r="G42" t="str">
         <f t="shared" si="0"/>
-        <v>40~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
@@ -900,7 +963,7 @@
       </c>
       <c r="G43" t="str">
         <f t="shared" si="0"/>
-        <v>41~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
@@ -910,7 +973,7 @@
       </c>
       <c r="G44" t="str">
         <f t="shared" si="0"/>
-        <v>42~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
@@ -920,7 +983,7 @@
       </c>
       <c r="G45" t="str">
         <f t="shared" si="0"/>
-        <v>43~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
@@ -930,7 +993,7 @@
       </c>
       <c r="G46" t="str">
         <f t="shared" si="0"/>
-        <v>44~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
@@ -940,7 +1003,7 @@
       </c>
       <c r="G47" t="str">
         <f t="shared" si="0"/>
-        <v>45~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
@@ -950,7 +1013,7 @@
       </c>
       <c r="G48" t="str">
         <f t="shared" si="0"/>
-        <v>46~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
@@ -960,7 +1023,7 @@
       </c>
       <c r="G49" t="str">
         <f t="shared" si="0"/>
-        <v>47~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
@@ -970,7 +1033,7 @@
       </c>
       <c r="G50" t="str">
         <f t="shared" si="0"/>
-        <v>48~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
@@ -980,7 +1043,7 @@
       </c>
       <c r="G51" t="str">
         <f t="shared" si="0"/>
-        <v>49~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
@@ -990,7 +1053,7 @@
       </c>
       <c r="G52" t="str">
         <f t="shared" si="0"/>
-        <v>50~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
@@ -1000,7 +1063,7 @@
       </c>
       <c r="G53" t="str">
         <f t="shared" si="0"/>
-        <v>51~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
@@ -1010,7 +1073,7 @@
       </c>
       <c r="G54" t="str">
         <f t="shared" si="0"/>
-        <v>52~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
@@ -1020,7 +1083,7 @@
       </c>
       <c r="G55" t="str">
         <f t="shared" si="0"/>
-        <v>53~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
@@ -1030,7 +1093,7 @@
       </c>
       <c r="G56" t="str">
         <f t="shared" si="0"/>
-        <v>54~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
@@ -1040,7 +1103,7 @@
       </c>
       <c r="G57" t="str">
         <f t="shared" si="0"/>
-        <v>55~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
@@ -1050,7 +1113,7 @@
       </c>
       <c r="G58" t="str">
         <f t="shared" si="0"/>
-        <v>56~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
@@ -1060,7 +1123,7 @@
       </c>
       <c r="G59" t="str">
         <f t="shared" si="0"/>
-        <v>57~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
@@ -1070,7 +1133,7 @@
       </c>
       <c r="G60" t="str">
         <f t="shared" si="0"/>
-        <v>58~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
@@ -1080,7 +1143,7 @@
       </c>
       <c r="G61" t="str">
         <f t="shared" si="0"/>
-        <v>59~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
@@ -1090,7 +1153,7 @@
       </c>
       <c r="G62" t="str">
         <f t="shared" si="0"/>
-        <v>60~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
@@ -1100,7 +1163,7 @@
       </c>
       <c r="G63" t="str">
         <f t="shared" si="0"/>
-        <v>61~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
@@ -1110,7 +1173,7 @@
       </c>
       <c r="G64" t="str">
         <f t="shared" si="0"/>
-        <v>62~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
@@ -1120,7 +1183,7 @@
       </c>
       <c r="G65" t="str">
         <f t="shared" si="0"/>
-        <v>63~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
@@ -1130,7 +1193,7 @@
       </c>
       <c r="G66" t="str">
         <f t="shared" si="0"/>
-        <v>64~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
@@ -1139,8 +1202,8 @@
         <v>65</v>
       </c>
       <c r="G67" t="str">
-        <f t="shared" ref="G67:G99" si="3">_xlfn.TEXTJOIN($H$7,FALSE,A67:F67)</f>
-        <v>65~~~~~</v>
+        <f t="shared" ref="G67:G99" si="3">IF(COUNT(B67:F67)&gt;0,_xlfn.TEXTJOIN($H$7,FALSE,A67:F67),"")</f>
+        <v/>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
@@ -1150,7 +1213,7 @@
       </c>
       <c r="G68" t="str">
         <f t="shared" si="3"/>
-        <v>66~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
@@ -1160,7 +1223,7 @@
       </c>
       <c r="G69" t="str">
         <f t="shared" si="3"/>
-        <v>67~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
@@ -1170,7 +1233,7 @@
       </c>
       <c r="G70" t="str">
         <f t="shared" si="3"/>
-        <v>68~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
@@ -1180,7 +1243,7 @@
       </c>
       <c r="G71" t="str">
         <f t="shared" si="3"/>
-        <v>69~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
@@ -1190,7 +1253,7 @@
       </c>
       <c r="G72" t="str">
         <f t="shared" si="3"/>
-        <v>70~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
@@ -1200,7 +1263,7 @@
       </c>
       <c r="G73" t="str">
         <f t="shared" si="3"/>
-        <v>71~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
@@ -1210,7 +1273,7 @@
       </c>
       <c r="G74" t="str">
         <f t="shared" si="3"/>
-        <v>72~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
@@ -1220,7 +1283,7 @@
       </c>
       <c r="G75" t="str">
         <f t="shared" si="3"/>
-        <v>73~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
@@ -1230,7 +1293,7 @@
       </c>
       <c r="G76" t="str">
         <f t="shared" si="3"/>
-        <v>74~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
@@ -1240,7 +1303,7 @@
       </c>
       <c r="G77" t="str">
         <f t="shared" si="3"/>
-        <v>75~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
@@ -1250,7 +1313,7 @@
       </c>
       <c r="G78" t="str">
         <f t="shared" si="3"/>
-        <v>76~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
@@ -1260,7 +1323,7 @@
       </c>
       <c r="G79" t="str">
         <f t="shared" si="3"/>
-        <v>77~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
@@ -1270,7 +1333,7 @@
       </c>
       <c r="G80" t="str">
         <f t="shared" si="3"/>
-        <v>78~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
@@ -1280,7 +1343,7 @@
       </c>
       <c r="G81" t="str">
         <f t="shared" si="3"/>
-        <v>79~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
@@ -1290,7 +1353,7 @@
       </c>
       <c r="G82" t="str">
         <f t="shared" si="3"/>
-        <v>80~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
@@ -1300,7 +1363,7 @@
       </c>
       <c r="G83" t="str">
         <f t="shared" si="3"/>
-        <v>81~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
@@ -1310,7 +1373,7 @@
       </c>
       <c r="G84" t="str">
         <f t="shared" si="3"/>
-        <v>82~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
@@ -1320,7 +1383,7 @@
       </c>
       <c r="G85" t="str">
         <f t="shared" si="3"/>
-        <v>83~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
@@ -1330,7 +1393,7 @@
       </c>
       <c r="G86" t="str">
         <f t="shared" si="3"/>
-        <v>84~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
@@ -1340,7 +1403,7 @@
       </c>
       <c r="G87" t="str">
         <f t="shared" si="3"/>
-        <v>85~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
@@ -1350,7 +1413,7 @@
       </c>
       <c r="G88" t="str">
         <f t="shared" si="3"/>
-        <v>86~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
@@ -1360,7 +1423,7 @@
       </c>
       <c r="G89" t="str">
         <f t="shared" si="3"/>
-        <v>87~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
@@ -1370,7 +1433,7 @@
       </c>
       <c r="G90" t="str">
         <f t="shared" si="3"/>
-        <v>88~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
@@ -1380,7 +1443,7 @@
       </c>
       <c r="G91" t="str">
         <f t="shared" si="3"/>
-        <v>89~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
@@ -1390,7 +1453,7 @@
       </c>
       <c r="G92" t="str">
         <f t="shared" si="3"/>
-        <v>90~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
@@ -1400,7 +1463,7 @@
       </c>
       <c r="G93" t="str">
         <f t="shared" si="3"/>
-        <v>91~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
@@ -1410,7 +1473,7 @@
       </c>
       <c r="G94" t="str">
         <f t="shared" si="3"/>
-        <v>92~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
@@ -1420,7 +1483,7 @@
       </c>
       <c r="G95" t="str">
         <f t="shared" si="3"/>
-        <v>93~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
@@ -1430,7 +1493,7 @@
       </c>
       <c r="G96" t="str">
         <f t="shared" si="3"/>
-        <v>94~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.3">
@@ -1440,7 +1503,7 @@
       </c>
       <c r="G97" t="str">
         <f t="shared" si="3"/>
-        <v>95~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.3">
@@ -1450,7 +1513,7 @@
       </c>
       <c r="G98" t="str">
         <f t="shared" si="3"/>
-        <v>96~~~~~</v>
+        <v/>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.3">
@@ -1460,7 +1523,7 @@
       </c>
       <c r="G99" t="str">
         <f t="shared" si="3"/>
-        <v>97~~~~~</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>